<commit_message>
Fix #205: rebuild example ADaM CSVs from clinTrialData CDISC pilot
Add data-raw/adam_example_data.R, which regenerates the example ADaM
CSVs in inst/extdata from clinTrialData's cdisc_pilot study, so the
test and example data have documented, reproducible provenance instead
of being hand-maintained. The data now follows pilot conventions
(TRT01AN 0/54/81, ISO dates), so the example ARS treatment conditions
and the affected test expectations are updated to match.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/extdata/exampleARS_3.xlsx
+++ b/inst/extdata/exampleARS_3.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="619" uniqueCount="619">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="622" uniqueCount="622">
   <si>
     <t>generatedUsing</t>
   </si>
@@ -1952,6 +1952,15 @@
   <si>
     <t xml:space="preserve">Mth_02_02_%_DEN</t>
   </si>
+  <si>
+    <t xml:space="preserve">54</t>
+  </si>
+  <si>
+    <t xml:space="preserve">81</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0</t>
+  </si>
 </sst>
 </file>
 
@@ -1970,7 +1979,6 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <b/>
     </font>
     <font>
@@ -1982,8 +1990,6 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
       <strike/>
     </font>
   </fonts>
@@ -5058,7 +5064,7 @@
         <v>234</v>
       </c>
       <c r="P2" t="s">
-        <v>309</v>
+        <v>619</v>
       </c>
     </row>
     <row r="3">
@@ -5099,7 +5105,7 @@
         <v>234</v>
       </c>
       <c r="P3" t="s">
-        <v>312</v>
+        <v>620</v>
       </c>
     </row>
     <row r="4">
@@ -5140,7 +5146,7 @@
         <v>234</v>
       </c>
       <c r="P4" t="s">
-        <v>315</v>
+        <v>621</v>
       </c>
     </row>
     <row r="5">
@@ -6121,7 +6127,7 @@
         <v>234</v>
       </c>
       <c r="P25" t="s">
-        <v>309</v>
+        <v>619</v>
       </c>
     </row>
     <row r="26">
@@ -6162,7 +6168,7 @@
         <v>234</v>
       </c>
       <c r="P26" t="s">
-        <v>312</v>
+        <v>620</v>
       </c>
     </row>
     <row r="27">
@@ -6203,7 +6209,7 @@
         <v>234</v>
       </c>
       <c r="P27" t="s">
-        <v>315</v>
+        <v>621</v>
       </c>
     </row>
     <row r="28">
@@ -6954,7 +6960,7 @@
         <v>234</v>
       </c>
       <c r="P44" t="s">
-        <v>309</v>
+        <v>619</v>
       </c>
     </row>
     <row r="45">
@@ -6995,7 +7001,7 @@
         <v>234</v>
       </c>
       <c r="P45" t="s">
-        <v>312</v>
+        <v>620</v>
       </c>
     </row>
     <row r="46">
@@ -7036,7 +7042,7 @@
         <v>234</v>
       </c>
       <c r="P46" t="s">
-        <v>315</v>
+        <v>621</v>
       </c>
     </row>
     <row r="47">
@@ -7602,7 +7608,7 @@
         <v>234</v>
       </c>
       <c r="P59" t="s">
-        <v>309</v>
+        <v>619</v>
       </c>
     </row>
     <row r="60">
@@ -7643,7 +7649,7 @@
         <v>234</v>
       </c>
       <c r="P60" t="s">
-        <v>312</v>
+        <v>620</v>
       </c>
     </row>
     <row r="61">
@@ -7684,7 +7690,7 @@
         <v>234</v>
       </c>
       <c r="P61" t="s">
-        <v>315</v>
+        <v>621</v>
       </c>
     </row>
     <row r="62">
@@ -8250,7 +8256,7 @@
         <v>234</v>
       </c>
       <c r="P74" t="s">
-        <v>309</v>
+        <v>619</v>
       </c>
     </row>
     <row r="75">
@@ -8291,7 +8297,7 @@
         <v>234</v>
       </c>
       <c r="P75" t="s">
-        <v>312</v>
+        <v>620</v>
       </c>
     </row>
     <row r="76">
@@ -8332,7 +8338,7 @@
         <v>234</v>
       </c>
       <c r="P76" t="s">
-        <v>315</v>
+        <v>621</v>
       </c>
     </row>
     <row r="77">

</xml_diff>

<commit_message>
Fix #205: use clinTrialData CDISC pilot as the only example ADaM source
Remove the bundled ADaM CSVs and their rebuild script; tests, examples and
vignettes now read the CDISC Pilot 01 ADaM from {clinTrialData}, and example
ARS fixtures use the pilot's own variable names. Tests that need data the
pilot lacks (RANDFL, COUNTRY, TRTDURM, ADEXSUM) skip until it is added
upstream rather than siera deriving it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/extdata/exampleARS_3.xlsx
+++ b/inst/extdata/exampleARS_3.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="622" uniqueCount="622">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="641" uniqueCount="641">
   <si>
     <t>generatedUsing</t>
   </si>
@@ -1960,6 +1960,63 @@
   </si>
   <si>
     <t xml:space="preserve">0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SEX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INTERSEX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RACE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMERICAN INDIAN OR ALASKA NATIVE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASIAN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BLACK OR AFRICAN AMERICAN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NATIVE HAWAIIAN OR OTHER PACIFIC ISLANDER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WHITE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OTHER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOT REPORTED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNKNOWN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ETHNIC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HISPANIC OR LATINO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOT HISPANIC OR LATINO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COUNTRY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USA</t>
   </si>
 </sst>
 </file>
@@ -5163,7 +5220,7 @@
         <v>225</v>
       </c>
       <c r="E5" t="s">
-        <v>319</v>
+        <v>622</v>
       </c>
       <c r="F5" t="s">
         <v>306</v>
@@ -5187,13 +5244,13 @@
         <v>225</v>
       </c>
       <c r="N5" t="s">
-        <v>319</v>
+        <v>622</v>
       </c>
       <c r="O5" t="s">
         <v>234</v>
       </c>
       <c r="P5" t="s">
-        <v>321</v>
+        <v>623</v>
       </c>
     </row>
     <row r="6">
@@ -5210,7 +5267,7 @@
         <v>225</v>
       </c>
       <c r="E6" t="s">
-        <v>319</v>
+        <v>622</v>
       </c>
       <c r="F6" t="s">
         <v>306</v>
@@ -5234,13 +5291,13 @@
         <v>225</v>
       </c>
       <c r="N6" t="s">
-        <v>319</v>
+        <v>622</v>
       </c>
       <c r="O6" t="s">
         <v>234</v>
       </c>
       <c r="P6" t="s">
-        <v>323</v>
+        <v>624</v>
       </c>
     </row>
     <row r="7">
@@ -5257,7 +5314,7 @@
         <v>225</v>
       </c>
       <c r="E7" t="s">
-        <v>319</v>
+        <v>622</v>
       </c>
       <c r="F7" t="s">
         <v>306</v>
@@ -5281,13 +5338,13 @@
         <v>225</v>
       </c>
       <c r="N7" t="s">
-        <v>319</v>
+        <v>622</v>
       </c>
       <c r="O7" t="s">
         <v>234</v>
       </c>
       <c r="P7" t="s">
-        <v>325</v>
+        <v>625</v>
       </c>
     </row>
     <row r="8">
@@ -5304,7 +5361,7 @@
         <v>225</v>
       </c>
       <c r="E8" t="s">
-        <v>319</v>
+        <v>622</v>
       </c>
       <c r="F8" t="s">
         <v>306</v>
@@ -5328,13 +5385,13 @@
         <v>225</v>
       </c>
       <c r="N8" t="s">
-        <v>319</v>
+        <v>622</v>
       </c>
       <c r="O8" t="s">
         <v>234</v>
       </c>
       <c r="P8" t="s">
-        <v>327</v>
+        <v>626</v>
       </c>
     </row>
     <row r="9">
@@ -5492,7 +5549,7 @@
         <v>225</v>
       </c>
       <c r="E12" t="s">
-        <v>342</v>
+        <v>627</v>
       </c>
       <c r="F12" t="s">
         <v>306</v>
@@ -5516,13 +5573,13 @@
         <v>225</v>
       </c>
       <c r="N12" t="s">
-        <v>342</v>
+        <v>627</v>
       </c>
       <c r="O12" t="s">
         <v>234</v>
       </c>
       <c r="P12" t="s">
-        <v>344</v>
+        <v>628</v>
       </c>
     </row>
     <row r="13">
@@ -5539,7 +5596,7 @@
         <v>225</v>
       </c>
       <c r="E13" t="s">
-        <v>342</v>
+        <v>627</v>
       </c>
       <c r="F13" t="s">
         <v>306</v>
@@ -5563,13 +5620,13 @@
         <v>225</v>
       </c>
       <c r="N13" t="s">
-        <v>342</v>
+        <v>627</v>
       </c>
       <c r="O13" t="s">
         <v>234</v>
       </c>
       <c r="P13" t="s">
-        <v>346</v>
+        <v>629</v>
       </c>
     </row>
     <row r="14">
@@ -5586,7 +5643,7 @@
         <v>225</v>
       </c>
       <c r="E14" t="s">
-        <v>342</v>
+        <v>627</v>
       </c>
       <c r="F14" t="s">
         <v>306</v>
@@ -5610,13 +5667,13 @@
         <v>225</v>
       </c>
       <c r="N14" t="s">
-        <v>342</v>
+        <v>627</v>
       </c>
       <c r="O14" t="s">
         <v>234</v>
       </c>
       <c r="P14" t="s">
-        <v>348</v>
+        <v>630</v>
       </c>
     </row>
     <row r="15">
@@ -5633,7 +5690,7 @@
         <v>225</v>
       </c>
       <c r="E15" t="s">
-        <v>342</v>
+        <v>627</v>
       </c>
       <c r="F15" t="s">
         <v>306</v>
@@ -5657,13 +5714,13 @@
         <v>225</v>
       </c>
       <c r="N15" t="s">
-        <v>342</v>
+        <v>627</v>
       </c>
       <c r="O15" t="s">
         <v>234</v>
       </c>
       <c r="P15" t="s">
-        <v>350</v>
+        <v>631</v>
       </c>
     </row>
     <row r="16">
@@ -5680,7 +5737,7 @@
         <v>225</v>
       </c>
       <c r="E16" t="s">
-        <v>342</v>
+        <v>627</v>
       </c>
       <c r="F16" t="s">
         <v>306</v>
@@ -5704,13 +5761,13 @@
         <v>225</v>
       </c>
       <c r="N16" t="s">
-        <v>342</v>
+        <v>627</v>
       </c>
       <c r="O16" t="s">
         <v>234</v>
       </c>
       <c r="P16" t="s">
-        <v>352</v>
+        <v>632</v>
       </c>
     </row>
     <row r="17">
@@ -5727,7 +5784,7 @@
         <v>225</v>
       </c>
       <c r="E17" t="s">
-        <v>342</v>
+        <v>627</v>
       </c>
       <c r="F17" t="s">
         <v>306</v>
@@ -5751,13 +5808,13 @@
         <v>225</v>
       </c>
       <c r="N17" t="s">
-        <v>342</v>
+        <v>627</v>
       </c>
       <c r="O17" t="s">
         <v>234</v>
       </c>
       <c r="P17" t="s">
-        <v>354</v>
+        <v>633</v>
       </c>
     </row>
     <row r="18">
@@ -5774,7 +5831,7 @@
         <v>225</v>
       </c>
       <c r="E18" t="s">
-        <v>342</v>
+        <v>627</v>
       </c>
       <c r="F18" t="s">
         <v>306</v>
@@ -5798,13 +5855,13 @@
         <v>225</v>
       </c>
       <c r="N18" t="s">
-        <v>342</v>
+        <v>627</v>
       </c>
       <c r="O18" t="s">
         <v>234</v>
       </c>
       <c r="P18" t="s">
-        <v>356</v>
+        <v>634</v>
       </c>
     </row>
     <row r="19">
@@ -5821,7 +5878,7 @@
         <v>225</v>
       </c>
       <c r="E19" t="s">
-        <v>342</v>
+        <v>627</v>
       </c>
       <c r="F19" t="s">
         <v>306</v>
@@ -5845,13 +5902,13 @@
         <v>225</v>
       </c>
       <c r="N19" t="s">
-        <v>342</v>
+        <v>627</v>
       </c>
       <c r="O19" t="s">
         <v>234</v>
       </c>
       <c r="P19" t="s">
-        <v>327</v>
+        <v>635</v>
       </c>
     </row>
     <row r="20">
@@ -5868,7 +5925,7 @@
         <v>225</v>
       </c>
       <c r="E20" t="s">
-        <v>361</v>
+        <v>636</v>
       </c>
       <c r="F20" t="s">
         <v>306</v>
@@ -5892,13 +5949,13 @@
         <v>225</v>
       </c>
       <c r="N20" t="s">
-        <v>361</v>
+        <v>636</v>
       </c>
       <c r="O20" t="s">
         <v>234</v>
       </c>
       <c r="P20" t="s">
-        <v>363</v>
+        <v>637</v>
       </c>
     </row>
     <row r="21">
@@ -5915,7 +5972,7 @@
         <v>225</v>
       </c>
       <c r="E21" t="s">
-        <v>361</v>
+        <v>636</v>
       </c>
       <c r="F21" t="s">
         <v>306</v>
@@ -5939,13 +5996,13 @@
         <v>225</v>
       </c>
       <c r="N21" t="s">
-        <v>361</v>
+        <v>636</v>
       </c>
       <c r="O21" t="s">
         <v>234</v>
       </c>
       <c r="P21" t="s">
-        <v>365</v>
+        <v>638</v>
       </c>
     </row>
     <row r="22">
@@ -5962,7 +6019,7 @@
         <v>225</v>
       </c>
       <c r="E22" t="s">
-        <v>361</v>
+        <v>636</v>
       </c>
       <c r="F22" t="s">
         <v>306</v>
@@ -5986,13 +6043,13 @@
         <v>225</v>
       </c>
       <c r="N22" t="s">
-        <v>361</v>
+        <v>636</v>
       </c>
       <c r="O22" t="s">
         <v>234</v>
       </c>
       <c r="P22" t="s">
-        <v>356</v>
+        <v>634</v>
       </c>
     </row>
     <row r="23">
@@ -6009,7 +6066,7 @@
         <v>225</v>
       </c>
       <c r="E23" t="s">
-        <v>361</v>
+        <v>636</v>
       </c>
       <c r="F23" t="s">
         <v>306</v>
@@ -6033,13 +6090,13 @@
         <v>225</v>
       </c>
       <c r="N23" t="s">
-        <v>361</v>
+        <v>636</v>
       </c>
       <c r="O23" t="s">
         <v>234</v>
       </c>
       <c r="P23" t="s">
-        <v>327</v>
+        <v>635</v>
       </c>
     </row>
     <row r="24">
@@ -6056,7 +6113,7 @@
         <v>225</v>
       </c>
       <c r="E24" t="s">
-        <v>371</v>
+        <v>639</v>
       </c>
       <c r="F24" t="s">
         <v>306</v>
@@ -6080,13 +6137,13 @@
         <v>225</v>
       </c>
       <c r="N24" t="s">
-        <v>371</v>
+        <v>639</v>
       </c>
       <c r="O24" t="s">
         <v>234</v>
       </c>
       <c r="P24" t="s">
-        <v>373</v>
+        <v>640</v>
       </c>
     </row>
     <row r="25">

</xml_diff>